<commit_message>
feat: add restricted platform public parser
</commit_message>
<xml_diff>
--- a/data/output/2026-05-28_实习信息.xlsx
+++ b/data/output/2026-05-28_实习信息.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y7"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="40" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
     <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
     <col width="31" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
@@ -978,13 +978,13 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Example Training</t>
+          <t>公开平台样例公司</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CAE 培训班招生</t>
+          <t>CAE 有限元仿真实习生</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -994,55 +994,59 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="H6" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>线上</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>暑期实习 3个月</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>CAE, Abaqus</t>
+          <t>CAE, 仿真, 结构分析, 有限元, Abaqus, Python</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Abaqus 培训班广告，非企业实习岗位</t>
+          <t>Abaqus Python 结构分析 暑期实习 3个月，参与真实研发项目。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>不建议优先投递：岗位与力学/机械/仿真研发方向匹配度不足或存在排除风险。</t>
+          <t>专业相关度高，命中 CAE、仿真、结构分析、有限元；技能匹配，涉及 Abaqus、Python；技术深度较好，包含 研发项目；成长性信号明确，出现 研发项目</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>疑似低相关或排除类岗位：培训班、广告</t>
+          <t>暂无明显风险</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>https://example.com/sample/training</t>
+          <t>https://example.com/sample/platform-cae</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>sample_manual</t>
+          <t>sample_platform_public</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1067,17 +1071,13 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sample Advanced Manufacturing</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>高端制造</t>
-        </is>
-      </c>
+          <t>Example Training</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>市场运营实习生</t>
+          <t>CAE 培训班招生</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1091,17 +1091,17 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>线上</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -1110,12 +1110,12 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>仿真</t>
+          <t>CAE, Abaqus</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>负责市场活动、销售支持和用户运营，不涉及研发或仿真。</t>
+          <t>Abaqus 培训班广告，非企业实习岗位</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>疑似低相关或排除类岗位：销售、市场、运营</t>
+          <t>疑似低相关或排除类岗位：培训班、广告</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>https://example.com/sample/marketing</t>
+          <t>https://example.com/sample/training</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>sample_static_html</t>
+          <t>sample_manual</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1151,6 +1151,99 @@
         </is>
       </c>
       <c r="Y7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sample Advanced Manufacturing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>高端制造</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>市场运营实习生</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CAE/有限元/结构仿真</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>仿真</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>负责市场活动、销售支持和用户运营，不涉及研发或仿真。</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>不建议优先投递：岗位与力学/机械/仿真研发方向匹配度不足或存在排除风险。</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>疑似低相关或排除类岗位：销售、市场、运营</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://example.com/sample/marketing</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>sample_static_html</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>